<commit_message>
Auto update ETF comparison: Fri Jul 10 09:39:59 UTC 2026
</commit_message>
<xml_diff>
--- a/data/00403A/20260709.xlsx
+++ b/data/00403A/20260709.xlsx
@@ -1423,14 +1423,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:E70"/>
   <sheetFormatPr defaultColWidth="8.43" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="24.9" bestFit="1" customWidth="1" collapsed="1"/>
-    <col min="2" max="2" width="24.75" bestFit="1" customWidth="1" collapsed="1"/>
-    <col min="3" max="3" width="12.9" bestFit="1" customWidth="1" collapsed="1"/>
-    <col min="4" max="4" width="10.35" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="1" max="1" width="24.9" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.75" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.9" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.35" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>